<commit_message>
Updated DSC Excel files, programme schedule template, and data records
</commit_message>
<xml_diff>
--- a/data/dsc_cane_scraping.xlsx
+++ b/data/dsc_cane_scraping.xlsx
@@ -1,20 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sibale\Desktop\Flask FarmManagementSystem\data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>Date</t>
   </si>
@@ -27,27 +32,12 @@
   <si>
     <t>Scrapers</t>
   </si>
-  <si>
-    <t>2025-06-03</t>
-  </si>
-  <si>
-    <t>2025-07-01</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>88</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -99,17 +89,26 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -156,7 +155,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -188,9 +187,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -222,6 +222,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -397,11 +398,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.7109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -415,32 +419,18 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
-      <c r="A2" t="s">
-        <v>4</v>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
+        <v>45748</v>
       </c>
       <c r="B2">
-        <v>1122</v>
+        <v>0</v>
       </c>
       <c r="C2">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="D2">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" t="s">
-        <v>8</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>